<commit_message>
multiple subs and project deactivate and activate
</commit_message>
<xml_diff>
--- a/Documents/Sub-lang-country-F2H26-Translation Document - SESAR.xlsx
+++ b/Documents/Sub-lang-country-F2H26-Translation Document - SESAR.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Adobe-Form-Builder-main\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C08C119D-DE1A-45AE-A724-6080DF29AF45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDC27046-D0CF-4729-815F-DA443A43B21C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="1710" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1812" yWindow="3816" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Complete Translations" sheetId="1" r:id="rId1"/>
     <sheet name="Samples" sheetId="5" r:id="rId2"/>
     <sheet name="Lists" sheetId="2" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="172">
   <si>
     <t>Translation</t>
   </si>
@@ -556,9 +556,6 @@
   </si>
   <si>
     <t>Project Code</t>
-  </si>
-  <si>
-    <t>F2H26</t>
   </si>
 </sst>
 </file>
@@ -1191,9 +1188,7 @@
       <c r="B2" t="s">
         <v>171</v>
       </c>
-      <c r="C2" s="17" t="s">
-        <v>172</v>
-      </c>
+      <c r="C2" s="17"/>
       <c r="D2" s="17"/>
     </row>
     <row r="3" spans="1:4" ht="15" thickBot="1">

</xml_diff>